<commit_message>
excel export for dasboard editor
</commit_message>
<xml_diff>
--- a/wtfmovies/public/excelTemplate/generalStatistical.xlsx
+++ b/wtfmovies/public/excelTemplate/generalStatistical.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\binhm\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\ruri\WTFmovies\wtfmovies\public\excelTemplate\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D629E1A-4095-46C5-81E3-2AF8A8F9F583}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A81BD08-90C8-4BC6-8BCE-1D3986D3BA90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{880F2132-E144-4513-B2A9-D12D5010211D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{880F2132-E144-4513-B2A9-D12D5010211D}"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="34">
   <si>
     <t>Views</t>
   </si>
@@ -125,17 +125,29 @@
   </si>
   <si>
     <t>Content</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Type/Month</t>
+  </si>
+  <si>
+    <t>Type/Year</t>
+  </si>
+  <si>
+    <t>2018</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -146,11 +158,26 @@
       <family val="1"/>
     </font>
     <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <b/>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -173,7 +200,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -182,21 +209,809 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="43">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="major"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -207,6 +1022,92 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{2821E573-AB6F-4BAE-8986-B1969B029559}" name="Table4" displayName="Table4" ref="A2:D4" totalsRowShown="0" headerRowDxfId="42" dataDxfId="41">
+  <autoFilter ref="A2:D4" xr:uid="{2821E573-AB6F-4BAE-8986-B1969B029559}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{4C5D4727-029F-4701-9CC3-83743C0D2483}" name="Type" dataDxfId="40"/>
+    <tableColumn id="2" xr3:uid="{4A2C3C58-6B0B-44E0-922C-14564D01601A}" name="Views" dataDxfId="39"/>
+    <tableColumn id="3" xr3:uid="{CD9A28DA-117B-4B35-BEC7-A2CAC6593DD0}" name="Users" dataDxfId="38"/>
+    <tableColumn id="4" xr3:uid="{08A94575-47F5-4FC9-B193-E9C4E5CEB39C}" name="Films" dataDxfId="37"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{5D21A084-4508-4FCA-8E73-F7981506BCB4}" name="Table5" displayName="Table5" ref="A7:M11" totalsRowShown="0" headerRowDxfId="36" dataDxfId="35">
+  <autoFilter ref="A7:M11" xr:uid="{5D21A084-4508-4FCA-8E73-F7981506BCB4}"/>
+  <tableColumns count="13">
+    <tableColumn id="1" xr3:uid="{AAF50735-7E8C-406D-AC0F-92A8B285B5E2}" name="Type/Month" dataDxfId="34"/>
+    <tableColumn id="2" xr3:uid="{8A31C595-B89F-42C3-A393-7CA3E7387FFC}" name="Jan" dataDxfId="33"/>
+    <tableColumn id="3" xr3:uid="{1314D8AF-09A1-4C73-94A6-EB1896418627}" name="Feb" dataDxfId="32"/>
+    <tableColumn id="4" xr3:uid="{DCFA11FA-6561-4A79-9AA8-2150782FC67C}" name="Mar" dataDxfId="31"/>
+    <tableColumn id="5" xr3:uid="{2813F2ED-8431-427C-8EE5-725DECE9A65C}" name="Apr" dataDxfId="30"/>
+    <tableColumn id="6" xr3:uid="{1CBB7B63-3DC5-4A47-B489-C7B5159BE797}" name="May" dataDxfId="29"/>
+    <tableColumn id="7" xr3:uid="{8C678A29-3C24-4288-901B-177E74B4BBF1}" name="Jun" dataDxfId="28"/>
+    <tableColumn id="8" xr3:uid="{708B939C-9B11-458F-A456-3E3B768DDC53}" name="Jul" dataDxfId="27"/>
+    <tableColumn id="9" xr3:uid="{09066E43-DE89-4EFB-8E2F-B9104401A6DA}" name="Aug" dataDxfId="26"/>
+    <tableColumn id="10" xr3:uid="{F414D160-50AA-445E-B138-B87A32D82B06}" name="Sep" dataDxfId="25"/>
+    <tableColumn id="11" xr3:uid="{7A15F18E-A4CC-4A36-BB09-E9F3520B88A9}" name="Oct" dataDxfId="24"/>
+    <tableColumn id="12" xr3:uid="{A5BF0AE9-E5E5-474C-A05A-126B1D926AF0}" name="Nov" dataDxfId="23"/>
+    <tableColumn id="13" xr3:uid="{CAA9D9E9-F490-4CE5-B677-8A3C4F3B1BF5}" name="Dec" dataDxfId="22"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{DE3F5CAB-4ABC-4F42-A78C-394119399905}" name="Table7" displayName="Table7" ref="A14:B17" totalsRowShown="0" headerRowDxfId="21">
+  <autoFilter ref="A14:B17" xr:uid="{DE3F5CAB-4ABC-4F42-A78C-394119399905}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{45158280-F594-4CAC-BFF5-2DBBE90B0C12}" name="Type/Year" dataDxfId="20"/>
+    <tableColumn id="2" xr3:uid="{4DA59E4D-1711-490B-98DF-40449AB08929}" name="2018" dataDxfId="19"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BA982284-1B43-403C-8027-C7CC59FBFFC8}" name="Table1" displayName="Table1" ref="A2:E7" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
+  <autoFilter ref="A2:E7" xr:uid="{BA982284-1B43-403C-8027-C7CC59FBFFC8}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{9C44FA24-C956-4690-85BE-0B524C776C43}" name="STT" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{86EE13A4-06DB-478F-BCF5-64B58957659D}" name="Name" dataDxfId="15"/>
+    <tableColumn id="3" xr3:uid="{CC2A241B-F033-4C46-8D0C-FFB237B50EEA}" name="Likes" dataDxfId="14"/>
+    <tableColumn id="4" xr3:uid="{9632C104-FBD0-4FB1-90C4-1AE5559F5BA6}" name="Views" dataDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{E4AB62C9-C618-4C3F-9C78-60FCD6E374C2}" name="Rating" dataDxfId="12"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{28AABA14-355E-48A9-9DFC-8FBFB6D18D33}" name="Table2" displayName="Table2" ref="A10:E14" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
+  <autoFilter ref="A10:E14" xr:uid="{28AABA14-355E-48A9-9DFC-8FBFB6D18D33}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{FDC42FCF-173E-4D14-8877-074980F1D44D}" name="STT" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{33249C9B-44E7-4595-94D4-E9545E50F55F}" name="Name" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{24F17C4B-924F-4FBF-BB97-8455D071CECA}" name="Likes" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{3337CD31-1EE1-4B4D-B7ED-F58D7F371918}" name="Views" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{EBC830E3-2F3A-47C0-A9C7-A937A7D5C598}" name="Rating" dataDxfId="5"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BB9D7677-864F-40B0-932B-DCEBAD5D19A4}" name="Table3" displayName="Table3" ref="A18:C23" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3">
+  <autoFilter ref="A18:C23" xr:uid="{BB9D7677-864F-40B0-932B-DCEBAD5D19A4}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{A25A1D1F-AC1B-4B5F-BB55-C02A3AD8FC08}" name="STT" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{2ACF4D46-3E48-4925-889C-34434915A3A0}" name="Content" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{690A52A7-536A-44BA-B26A-C36698D2321B}" name="Times" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -507,18 +1408,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E071C786-B8C3-46DA-BCB8-6F6F4FD72D86}">
   <dimension ref="A1:M17"/>
-  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.8984375" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="2" customWidth="1"/>
-    <col min="2" max="16384" width="8.88671875" style="1"/>
+    <col min="1" max="1" width="12.19921875" style="2" customWidth="1"/>
+    <col min="2" max="16384" width="8.8984375" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="7" t="s">
         <v>20</v>
       </c>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>30</v>
+      </c>
       <c r="B2" s="3" t="s">
         <v>0</v>
       </c>
@@ -540,11 +1447,26 @@
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="7" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="7" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="7"/>
+      <c r="C6" s="7"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="7"/>
+      <c r="G6" s="7"/>
+      <c r="H6" s="7"/>
+      <c r="I6" s="7"/>
+      <c r="J6" s="7"/>
+      <c r="K6" s="7"/>
+      <c r="L6" s="7"/>
+      <c r="M6" s="7"/>
+    </row>
+    <row r="7" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>31</v>
+      </c>
       <c r="B7" s="2" t="s">
         <v>5</v>
       </c>
@@ -597,14 +1519,18 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A12" s="4" t="s">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A13" s="7" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="14" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="2">
-        <v>2018</v>
+      <c r="B13" s="7"/>
+    </row>
+    <row r="14" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.3">
@@ -623,159 +1549,189 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A6:M6"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="3">
+    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
+  </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16008A9C-77FE-4229-B954-E8AE76D02E4C}">
   <dimension ref="A1:E23"/>
-  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.8984375" defaultRowHeight="16.8" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="5"/>
-    <col min="2" max="2" width="35.33203125" style="5" customWidth="1"/>
-    <col min="3" max="16384" width="8.88671875" style="5"/>
+    <col min="1" max="1" width="16.09765625" style="4" customWidth="1"/>
+    <col min="2" max="2" width="35.296875" style="4" customWidth="1"/>
+    <col min="3" max="16384" width="8.8984375" style="4"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="8" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="6" t="s">
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+    </row>
+    <row r="2" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="5" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="7">
+      <c r="A3" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" s="7">
+      <c r="A4" s="6">
         <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="7">
+      <c r="A5" s="6">
         <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" s="7">
+      <c r="A6" s="6">
         <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" s="7">
+      <c r="A7" s="6">
         <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="8" t="s">
         <v>26</v>
       </c>
+      <c r="B9" s="8"/>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="D10" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="E10" s="5" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" s="5">
+      <c r="A11" s="4">
         <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" s="5">
+      <c r="A12" s="4">
         <v>2</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A13" s="5">
+      <c r="A13" s="4">
         <v>3</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" s="5">
+      <c r="A14" s="4">
         <v>4</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" s="5">
+      <c r="A15" s="4">
         <v>5</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="5" t="s">
+      <c r="A17" s="8" t="s">
         <v>27</v>
       </c>
+      <c r="B17" s="8"/>
+      <c r="C17" s="8"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="6" t="s">
+      <c r="A18" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="B18" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="C18" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="D18" s="6"/>
-      <c r="E18" s="6"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A19" s="5">
+      <c r="A19" s="4">
         <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A20" s="5">
+      <c r="A20" s="4">
         <v>2</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A21" s="5">
+      <c r="A21" s="4">
         <v>3</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A22" s="5">
+      <c r="A22" s="4">
         <v>4</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A23" s="5">
+      <c r="A23" s="4">
         <v>5</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A9:E9"/>
+    <mergeCell ref="A17:C17"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <tableParts count="3">
+    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId4"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>